<commit_message>
Updated dashboard and PostgreSQL integration
</commit_message>
<xml_diff>
--- a/north_is_jobs_analysis.xlsx
+++ b/north_is_jobs_analysis.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,7 +480,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>75</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -499,7 +499,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>מיישם/ת מערכות מידע המכללה האקדמית להנדסה בראודה כרמיאל | 3-4 שנים | משרה מלאה | לפני 22 שעות למחלקת טכנולוגיות מידע  דרוש/ה מיישם/ת מערכות מידע    תכולת התפקיד :  מתן שירות תמיכה והטמ... + לצפייה בפרטי המשרה</t>
+          <t>מיישם/ת מערכות מידע המכללה האקדמית להנדסה בראודה כרמיאל | 3-4 שנים | משרה מלאה | לפני 6 שעות למחלקת טכנולוגיות מידע  דרוש/ה מיישם/ת מערכות מידע    תכולת התפקיד :  מתן שירות תמיכה והטמ... + לצפייה בפרטי המשרה</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -511,7 +511,7 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://www.drushim.co.il/jobs/search/מיישם%20מערכות%20מידע/</t>
+          <t>https://www.drushim.co.il/jobs/search/מערכות%20מידע/</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -530,7 +530,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>76</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -580,7 +580,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>77</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -630,7 +630,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>78</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -680,11 +680,11 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>79</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>מידענ.ית לצוות בקרת תצורה פורסם לפני 1 שעות ע"י אלביט מערכות בע"מ כרמיאל משרה מל</t>
+          <t>בוגר/ת מערכות מידע- משרה התחלתית פורסם לפני 8 שעות ע"י גב אקספרט חיפה משרה מלאה</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -699,13 +699,13 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>מידענ.ית לצוות בקרת תצורה פורסם לפני 1 שעות ע"י אלביט מערכות בע"מ כרמיאל משרה מלאה We are looking for
-our Elbit Cyclone site in Bar-Lev Industrial Zone, we are looking for a Configuration Control Specialist to join our team. In this role, you ... הגש מועמדות שמור למועדפים משרות נוספות</t>
+          <t>בוגר/ת מערכות מידע- משרה התחלתית פורסם לפני 8 שעות ע"י גב אקספרט חיפה משרה מלאה אקדמאים ללא נסיון, ללא נסיון התואר במערכות מידע ביד ואתם מחפשים את המקום שבו תהפכו את התיאוריה לפרקטיקה?
+אנחנו מחפשים מיישם/ת ומפתח/ת מערכות ITSM לתפקיד התחלתי (Junior). אם אתם רוצים לצמוח ... הגש מועמדות שמור למועדפים משרות נוספות</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>BI</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -731,12 +731,11 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>כרמיאל משרה מלאה We are looking for
-our Elbit Cyclone site in Bar-Lev Industrial</t>
+          <t>חיפה משרה מלאה אקדמאים ללא נסיון, ללא נסיון התואר במערכות מידע ביד ואתם מחפשים א</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -751,13 +750,13 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>כרמיאל משרה מלאה We are looking for
-our Elbit Cyclone site in Bar-Lev Industrial Zone, we are looking for a Configuration Control Specialist to join our team. In this role, you ...</t>
+          <t>חיפה משרה מלאה אקדמאים ללא נסיון, ללא נסיון התואר במערכות מידע ביד ואתם מחפשים את המקום שבו תהפכו את התיאוריה לפרקטיקה?
+אנחנו מחפשים מיישם/ת ומפתח/ת מערכות ITSM לתפקיד התחלתי (Junior). אם אתם רוצים לצמוח ...</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>BI</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -783,11 +782,11 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
+        <v>81</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ראש.ת צוות מערכות מידע פורסם לפני 1 שעות ע"י אלביט מערכות בע"מ חיפה משרה מלאה אנ</t>
+          <t>מיישם/ת Priority ומנהל/ת פרויקטי מערכות מידע - קריית גת פורסם לפני 8 שעות ע"י תי</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -802,28 +801,28 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ראש.ת צוות מערכות מידע פורסם לפני 1 שעות ע"י אלביט מערכות בע"מ חיפה משרה מלאה אנחנו מגייסים ראש.ת צוות מערכות מידע מנוסה להובלת צוות פיתוח בתחום PLM באתר החברה בחיפה.
-אם יש לך תשוקה לטכנולוגיה, ניסיון בניהול צוותים, ורצון להשפיע על מערכו... הגש מועמדות שמור למועדפים משרות נוספות</t>
+          <t>מיישם/ת Priority ומנהל/ת פרויקטי מערכות מידע - קריית גת פורסם לפני 8 שעות ע"י תיגבור חברה ארצית לשרותי כ"א קריית גת משרה מלאה מיישם/ת Priority ומנהל/ת פרויקטי מערכות מידע
+ הובלת פרויקטי מחשוב מקצה לקצה. עבודה עם מערכות ארגוניות מתקדמות. שיפור תהליכים, הטמעה וליווי משתמשים. שילוב פתרונ... הגש מועמדות שמור למועדפים משרות נוספות</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>מערכות מידע</t>
+          <t>מערכות מידע, Priority</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://www.jobmaster.co.il/jobs/?q=מערכות+מידע</t>
+          <t>https://www.jobmaster.co.il/jobs/?q=מיישם+מערכות+מידע</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>התאמה נמוכה</t>
+          <t>התאמה בינונית</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -834,11 +833,12 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>8</v>
+        <v>82</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>חיפה משרה מלאה אנחנו מגייסים ראש.ת צוות מערכות מידע מנוסה להובלת צוות פיתוח בתחו</t>
+          <t>קריית גת משרה מלאה מיישם/ת Priority ומנהל/ת פרויקטי מערכות מידע
+ הובלת פרויקטי</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -853,28 +853,28 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>חיפה משרה מלאה אנחנו מגייסים ראש.ת צוות מערכות מידע מנוסה להובלת צוות פיתוח בתחום PLM באתר החברה בחיפה.
-אם יש לך תשוקה לטכנולוגיה, ניסיון בניהול צוותים, ורצון להשפיע על מערכו...</t>
+          <t>קריית גת משרה מלאה מיישם/ת Priority ומנהל/ת פרויקטי מערכות מידע
+ הובלת פרויקטי מחשוב מקצה לקצה. עבודה עם מערכות ארגוניות מתקדמות. שיפור תהליכים, הטמעה וליווי משתמשים. שילוב פתרונ...</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>מערכות מידע</t>
+          <t>מערכות מידע, Priority</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://www.jobmaster.co.il/jobs/?q=מערכות+מידע</t>
+          <t>https://www.jobmaster.co.il/jobs/?q=מיישם+מערכות+מידע</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>התאמה נמוכה</t>
+          <t>התאמה בינונית</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -885,11 +885,11 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>9</v>
+        <v>83</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>דרוש/ה מיישמ/ת מערכות מידע אלקטרוניות פורסם לפני 5 שעות ע"י אי.אס טופ פרוג’קטס ב</t>
+          <t>מיישם/ת Priority ומנהל/ת פרויקטי מערכות מידע פורסם לפני 8 שעות ע"י תיגבור חברה א</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -904,14 +904,13 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>דרוש/ה מיישמ/ת מערכות מידע אלקטרוניות פורסם לפני 5 שעות ע"י אי.אס טופ פרוג’קטס בע"מ קריית ים משרה מלאה לאי אס טופ פרוג’קטס דרוש/ה מיישמ/ת מערכות מידע אלקטרוניות.
-התפקיד כולל:
-- מתן מענה בנושא IT למהנדסי פיתוח אלקטרוניקה בכלי CAD אלקטרוניים (תכן, עריכה, סי... הגש מועמדות שמור למועדפים משרות נוספות</t>
+          <t>מיישם/ת Priority ומנהל/ת פרויקטי מערכות מידע פורסם לפני 8 שעות ע"י תיגבור חברה ארצית לשרותי כ"א קריית גת משרה מלאה מיישם/ת Priority ומנהל/ת פרויקטי מערכות מידע
+הצטרפות לצוות מערכות המידע של הארגון. הובלת פרויקטי מחשוב מקצה לקצה. עבודה עם מערכות ארגוניות מתקדמות. שיפור תהליכ... הגש מועמדות שמור למועדפים משרות נוספות</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>מערכות מידע</t>
+          <t>מערכות מידע, Priority</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -922,11 +921,11 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>התאמה נמוכה</t>
+          <t>התאמה בינונית</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -937,140 +936,138 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>10</v>
+        <v>84</v>
       </c>
       <c r="B11" t="inlineStr">
+        <is>
+          <t>קריית גת משרה מלאה מיישם/ת Priority ומנהל/ת פרויקטי מערכות מידע
+הצטרפות לצוות מ</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>צפון / לבדוק במודעה</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>קריית גת משרה מלאה מיישם/ת Priority ומנהל/ת פרויקטי מערכות מידע
+הצטרפות לצוות מערכות המידע של הארגון. הובלת פרויקטי מחשוב מקצה לקצה. עבודה עם מערכות ארגוניות מתקדמות. שיפור תהליכ...</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>מערכות מידע, Priority</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://www.jobmaster.co.il/jobs/?q=מיישם+מערכות+מידע</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>40</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>התאמה בינונית</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>JobMaster</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>85</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>דרוש/ה מיישמ/ת מערכות מידע אלקטרוניות פורסם לפני 14 שעות ע"י אי.אס טופ פרוג’קטס</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>צפון / לבדוק במודעה</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>דרוש/ה מיישמ/ת מערכות מידע אלקטרוניות פורסם לפני 14 שעות ע"י אי.אס טופ פרוג’קטס בע"מ קריית ים משרה מלאה לאי אס טופ פרוג’קטס דרוש/ה מיישמ/ת מערכות מידע אלקטרוניות.
+התפקיד כולל:
+- מתן מענה בנושא IT למהנדסי פיתוח אלקטרוניקה בכלי CAD אלקטרוניים (תכן, עריכה, סי... הגש מועמדות שמור למועדפים משרות נוספות</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>מערכות מידע</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://www.jobmaster.co.il/jobs/?q=מיישם+מערכות+מידע</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>20</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>התאמה נמוכה</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>JobMaster</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>86</v>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>קריית ים משרה מלאה לאי אס טופ פרוג’קטס דרוש/ה מיישמ/ת מערכות מידע אלקטרוניות.
 ה</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>לא ידוע</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>צפון / לבדוק במודעה</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>צפון / לבדוק במודעה</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>קריית ים משרה מלאה לאי אס טופ פרוג’קטס דרוש/ה מיישמ/ת מערכות מידע אלקטרוניות.
 התפקיד כולל:
 - מתן מענה בנושא IT למהנדסי פיתוח אלקטרוניקה בכלי CAD אלקטרוניים (תכן, עריכה, סי...</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>מערכות מידע</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>https://www.jobmaster.co.il/jobs/?q=מיישם+מערכות+מידע</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
-        <v>20</v>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>התאמה נמוכה</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>JobMaster</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>לחברה תעשייתית דרוש/ה מיישם/ת מערכות מידע פורסם לפני 6 שעות ע"י שרון גרינברג כרמ</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>לא ידוע</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>צפון / לבדוק במודעה</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>לחברה תעשייתית דרוש/ה מיישם/ת מערכות מידע פורסם לפני 6 שעות ע"י שרון גרינברג כרמיאל, מעלות תרשיחא, נהריה, עכו, צפת משרה מלאה משרה בכירה לחברה תעשייתית דרוש/ה מיישם/ת מערכות מידע
--ניסיון כמיישם/ת מערכות ERP - חובה!
--ניסיון במערכת WMS - יתרון!
-השכלה רלוונטית הגש מועמדות שמור למועדפים משרות נוספות</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>מערכות מידע, ERP</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>https://www.jobmaster.co.il/jobs/?q=מיישם+מערכות+מידע</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
-        <v>40</v>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>התאמה בינונית</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>JobMaster</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>כרמיאל, מעלות תרשיחא, נהריה, עכו, צפת משרה מלאה משרה בכירה לחברה תעשייתית דרוש/ה</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>לא ידוע</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>צפון / לבדוק במודעה</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>כרמיאל, מעלות תרשיחא, נהריה, עכו, צפת משרה מלאה משרה בכירה לחברה תעשייתית דרוש/ה מיישם/ת מערכות מידע
--ניסיון כמיישם/ת מערכות ERP - חובה!
--ניסיון במערכת WMS - יתרון!
-השכלה רלוונטית</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>מערכות מידע, ERP</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
@@ -1081,11 +1078,11 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>התאמה בינונית</t>
+          <t>התאמה נמוכה</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1096,11 +1093,11 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>13</v>
+        <v>87</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>מיישם/ת Priority ומנהל/ת פרויקטי מערכות מידע פורסם לפני 1 ימים ע"י תיגבור חברה א</t>
+          <t>מיישם/ת  ERP Priority פורסם לפני 10 שעות ע"י קבוצת עפיפי טכנולוגיות תחבורה ותייר</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1115,20 +1112,20 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>מיישם/ת Priority ומנהל/ת פרויקטי מערכות מידע פורסם לפני 1 ימים ע"י תיגבור חברה ארצית לשרותי כ"א קריית גת משרה מלאה מיישם/ת Priority ומנהל/ת פרויקטי מערכות מידע
-הצטרפות לצוות מערכות המידע של הארגון. הובלת פרויקטי מחשוב מקצה לקצה. עבודה עם מערכות ארגוניות מתקדמות. שיפור תהליכ... הגש מועמדות שמור למועדפים משרות נוספות</t>
+          <t>מיישם/ת  ERP Priority פורסם לפני 10 שעות ע"י קבוצת עפיפי טכנולוגיות תחבורה ותיירות נצרת משרה מלאה מיישם/ת  ERP Priority 
+אפסילון דלתא, חברה מובילה בתחום המכונאות, היבוא והסחר, מגייסת מיישם/ת ERP למחלקת ה-IT. התפקיד כולל הובלת פרויקטים חוצי ארגון, הטמעת מערכ... הגש מועמדות שמור למועדפים משרות נוספות</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>מערכות מידע, Priority</t>
+          <t>ERP, Priority</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://www.jobmaster.co.il/jobs/?q=מיישם+מערכות+מידע</t>
+          <t>https://www.jobmaster.co.il/jobs/?q=ERP</t>
         </is>
       </c>
       <c r="J14" t="n">
@@ -1147,12 +1144,12 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>14</v>
+        <v>88</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>קריית גת משרה מלאה מיישם/ת Priority ומנהל/ת פרויקטי מערכות מידע
-הצטרפות לצוות מ</t>
+          <t>נצרת משרה מלאה מיישם/ת  ERP Priority 
+אפסילון דלתא, חברה מובילה בתחום המכונאות,</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1167,20 +1164,20 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>קריית גת משרה מלאה מיישם/ת Priority ומנהל/ת פרויקטי מערכות מידע
-הצטרפות לצוות מערכות המידע של הארגון. הובלת פרויקטי מחשוב מקצה לקצה. עבודה עם מערכות ארגוניות מתקדמות. שיפור תהליכ...</t>
+          <t>נצרת משרה מלאה מיישם/ת  ERP Priority 
+אפסילון דלתא, חברה מובילה בתחום המכונאות, היבוא והסחר, מגייסת מיישם/ת ERP למחלקת ה-IT. התפקיד כולל הובלת פרויקטים חוצי ארגון, הטמעת מערכ...</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>מערכות מידע, Priority</t>
+          <t>ERP, Priority</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://www.jobmaster.co.il/jobs/?q=מיישם+מערכות+מידע</t>
+          <t>https://www.jobmaster.co.il/jobs/?q=ERP</t>
         </is>
       </c>
       <c r="J15" t="n">
@@ -1199,11 +1196,11 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>15</v>
+        <v>89</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>מיישם/ת  ERP Priority פורסם לפני 1 שעות ע"י קבוצת עפיפי טכנולוגיות תחבורה ותיירו</t>
+          <t>מיישם ERP לחברת טיפוח בינלאומית מובילה בצפון פורסם לפני 10 שעות ע"י גפן השמות כר</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1218,13 +1215,14 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>מיישם/ת  ERP Priority פורסם לפני 1 שעות ע"י קבוצת עפיפי טכנולוגיות תחבורה ותיירות נצרת משרה מלאה מיישם/ת  ERP Priority 
-אפסילון דלתא, חברה מובילה בתחום המכונאות, היבוא והסחר, מגייסת מיישם/ת ERP למחלקת ה-IT. התפקיד כולל הובלת פרויקטים חוצי ארגון, הטמעת מערכ... הגש מועמדות שמור למועדפים משרות נוספות</t>
+          <t>מיישם ERP לחברת טיפוח בינלאומית מובילה בצפון פורסם לפני 10 שעות ע"י גפן השמות כרמיאל משרה מלאה עבודה היברידית תפקידים ואחריות:
+• השתתפות בהטמעת פרויקט ארגוני רחב היקף של ERP + WMS.
+• השתתפות בניהול פרויקטים מקצה לקצה (End-to-End), כולל אפיון תהליכים, הגדרה, יישום, בדיקו... הגש מועמדות שמור למועדפים משרות נוספות</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>ERP, Priority</t>
+          <t>ERP, אפיון</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -1250,12 +1248,12 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>16</v>
+        <v>90</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>נצרת משרה מלאה מיישם/ת  ERP Priority 
-אפסילון דלתא, חברה מובילה בתחום המכונאות,</t>
+          <t>כרמיאל משרה מלאה עבודה היברידית תפקידים ואחריות:
+• השתתפות בהטמעת פרויקט ארגוני</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1270,13 +1268,14 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>נצרת משרה מלאה מיישם/ת  ERP Priority 
-אפסילון דלתא, חברה מובילה בתחום המכונאות, היבוא והסחר, מגייסת מיישם/ת ERP למחלקת ה-IT. התפקיד כולל הובלת פרויקטים חוצי ארגון, הטמעת מערכ...</t>
+          <t>כרמיאל משרה מלאה עבודה היברידית תפקידים ואחריות:
+• השתתפות בהטמעת פרויקט ארגוני רחב היקף של ERP + WMS.
+• השתתפות בניהול פרויקטים מקצה לקצה (End-to-End), כולל אפיון תהליכים, הגדרה, יישום, בדיקו...</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>ERP, Priority</t>
+          <t>ERP, אפיון</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
@@ -1295,268 +1294,6 @@
         </is>
       </c>
       <c r="L17" t="inlineStr">
-        <is>
-          <t>JobMaster</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>מיישם ERP לחברת טיפוח בינלאומית מובילה בצפון פורסם לפני 1 שעות ע"י גפן השמות כרמ</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>לא ידוע</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>צפון / לבדוק במודעה</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>מיישם ERP לחברת טיפוח בינלאומית מובילה בצפון פורסם לפני 1 שעות ע"י גפן השמות כרמיאל משרה מלאה עבודה היברידית תפקידים ואחריות:
-• השתתפות בהטמעת פרויקט ארגוני רחב היקף של ERP + WMS.
-• השתתפות בניהול פרויקטים מקצה לקצה (End-to-End), כולל אפיון תהליכים, הגדרה, יישום, בדיקו... הגש מועמדות שמור למועדפים משרות נוספות</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>ERP, אפיון</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>https://www.jobmaster.co.il/jobs/?q=ERP</t>
-        </is>
-      </c>
-      <c r="J18" t="n">
-        <v>40</v>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>התאמה בינונית</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>JobMaster</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>כרמיאל משרה מלאה עבודה היברידית תפקידים ואחריות:
-• השתתפות בהטמעת פרויקט ארגוני</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>לא ידוע</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>צפון / לבדוק במודעה</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>כרמיאל משרה מלאה עבודה היברידית תפקידים ואחריות:
-• השתתפות בהטמעת פרויקט ארגוני רחב היקף של ERP + WMS.
-• השתתפות בניהול פרויקטים מקצה לקצה (End-to-End), כולל אפיון תהליכים, הגדרה, יישום, בדיקו...</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>ERP, אפיון</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>https://www.jobmaster.co.il/jobs/?q=ERP</t>
-        </is>
-      </c>
-      <c r="J19" t="n">
-        <v>40</v>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>התאמה בינונית</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>JobMaster</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>דרוש/ה מפתח/ת BI פורסם לפני 5 שעות ע"י אי.אס טופ פרוג’קטס בע"מ חיפה משרה מלאה לא</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>לא ידוע</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>צפון / לבדוק במודעה</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>דרוש/ה מפתח/ת BI פורסם לפני 5 שעות ע"י אי.אס טופ פרוג’קטס בע"מ חיפה משרה מלאה לאי אס טופ פרוג’טס דרוש/ה מפתח/ת BI מנוסה לעבודה במפעל בטחוני גדול בצפון.
-התפקיד כולל:
-- פיתוח ויישום פתרונות BI מתקדמים ותובנות עסקיות מנתונים מורכבים.... הגש מועמדות שמור למועדפים משרות נוספות</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>BI</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>https://www.jobmaster.co.il/jobs/?q=BI</t>
-        </is>
-      </c>
-      <c r="J20" t="n">
-        <v>20</v>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>התאמה נמוכה</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>JobMaster</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>חיפה משרה מלאה לאי אס טופ פרוג’טס דרוש/ה מפתח/ת BI מנוסה לעבודה במפעל בטחוני גדו</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>לא ידוע</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>צפון / לבדוק במודעה</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>חיפה משרה מלאה לאי אס טופ פרוג’טס דרוש/ה מפתח/ת BI מנוסה לעבודה במפעל בטחוני גדול בצפון.
-התפקיד כולל:
-- פיתוח ויישום פתרונות BI מתקדמים ותובנות עסקיות מנתונים מורכבים....</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>BI</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>https://www.jobmaster.co.il/jobs/?q=BI</t>
-        </is>
-      </c>
-      <c r="J21" t="n">
-        <v>20</v>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>התאמה נמוכה</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>JobMaster</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>לאי אס טופ פרוג’טס דרוש/ה מפתח/ת BI מנוסה לעבודה במפעל בטחוני גדול בצפון.
-התפקי</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>לא ידוע</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>צפון / לבדוק במודעה</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>לאי אס טופ פרוג’טס דרוש/ה מפתח/ת BI מנוסה לעבודה במפעל בטחוני גדול בצפון.
-התפקיד כולל:
-- פיתוח ויישום פתרונות BI מתקדמים ותובנות עסקיות מנתונים מורכבים....</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>BI</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>https://www.jobmaster.co.il/jobs/?q=BI</t>
-        </is>
-      </c>
-      <c r="J22" t="n">
-        <v>20</v>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>התאמה נמוכה</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
         <is>
           <t>JobMaster</t>
         </is>

</xml_diff>